<commit_message>
Finalize competitor ads sheet: add second Nowwin ad (16 ads)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDCiezjHZtSKU1uv8fZ38q
</commit_message>
<xml_diff>
--- a/deliverables/Zarthi_Competitor_Meta_Ads_India.xlsx
+++ b/deliverables/Zarthi_Competitor_Meta_Ads_India.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Takeaways for Zarthi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Competitor Ads'!$A$4:$N$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Competitor Ads'!$A$4:$N$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -554,14 +554,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Zarthi · Cloud Architect hiring · Meta Ad Library scan (India, active ads)</t>
+          <t>Zarthi · Cloud Architect hiring · Meta Ad Library scan (India, active ads) · FINAL</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pulled 28 Sep 2026 from Meta Ad Library, filtered to ads delivered in India, active, paid in INR. Yellow columns (Caption, Description, CTA) are not returned by Meta's Ad Library tool: open the Ad Library link in each row and copy them in.</t>
+          <t>Pulled 28 Sep 2026 from Meta Ad Library, filtered to ads delivered in India, active, paid in INR. Caption, Description and CTA (yellow) are not returned by Meta's Ad Library tool, and facebook.com is blocked from this environment. Open the link in each row to view them.</t>
         </is>
       </c>
     </row>
@@ -704,38 +704,38 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Iconic Options</t>
+          <t>Nowwin Technologies</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>1022000921003672</t>
+          <t>851245194944831</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>1142990505055359</t>
+          <t>4506695909546073</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Hiring IT Professionals | 6–8 Years</t>
+          <t>10+ Years PeopleSoft Experience? Apply Now</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr"/>
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="7" t="n">
-        <v>46292.89021990741</v>
+        <v>46290.00069444445</v>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>Mid-senior IT professionals</t>
+          <t>Senior (10+ yr) enterprise-tech specialists</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Experience call-out</t>
+          <t>Experience call-out (10+ years, same as Zarthi's plan)</t>
         </is>
       </c>
       <c r="M6" s="8" t="inlineStr">
@@ -760,38 +760,38 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Prism IT Hub</t>
+          <t>Iconic Options</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>1042916842245951</t>
+          <t>1022000921003672</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>1570863821744505</t>
+          <t>1142990505055359</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>TCS Hiring | 6+ Years | Apply Now</t>
+          <t>Hiring IT Professionals | 6–8 Years</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr"/>
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="7" t="n">
-        <v>46291.6772337963</v>
+        <v>46292.89021990741</v>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>Experienced IT services staff (likely third-party recruiter using a big employer name)</t>
+          <t>Mid-senior IT professionals</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Big-brand borrowing + experience</t>
+          <t>Experience call-out</t>
         </is>
       </c>
       <c r="M7" s="8" t="inlineStr">
@@ -816,38 +816,38 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>hirist.tech</t>
+          <t>Prism IT Hub</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>446429982057859</t>
+          <t>1042916842245951</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>1424325016466491</t>
+          <t>1570863821744505</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>ARMPL / Solution Analysts / Clovio IT Consulting / Scout Incorporation / Career Infosystem / Happiest Minds Technologies is hiring | Apply now</t>
+          <t>TCS Hiring | 6+ Years | Apply Now</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="7" t="n">
-        <v>46273.84724537037</v>
+        <v>46291.6772337963</v>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Indian tech professionals (job board, rotates employers)</t>
+          <t>Experienced IT services staff (likely third-party recruiter using a big employer name)</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Multi-employer job feed</t>
+          <t>Big-brand borrowing + experience</t>
         </is>
       </c>
       <c r="M8" s="8" t="inlineStr">
@@ -872,38 +872,38 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>FPA AI</t>
+          <t>hirist.tech</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>1412353528623168</t>
+          <t>446429982057859</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>28796808946621878</t>
+          <t>1424325016466491</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>FPA AI | Enterprise Technology &amp; AI Advisory | Join US! | In Digital Transformation | Of Our Offerings | Scan QR</t>
+          <t>ARMPL / Solution Analysts / Clovio IT Consulting / Scout Incorporation / Career Infosystem / Happiest Minds Technologies is hiring | Apply now</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr"/>
       <c r="H9" s="6" t="inlineStr"/>
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="7" t="n">
-        <v>46292.20268518518</v>
+        <v>46273.84724537037</v>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Consulting / architecture talent (closest match to Zarthi)</t>
+          <t>Indian tech professionals (job board, rotates employers)</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Employer brand + offerings</t>
+          <t>Multi-employer job feed</t>
         </is>
       </c>
       <c r="M9" s="8" t="inlineStr">
@@ -928,38 +928,38 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Exano Technologies</t>
+          <t>FPA AI</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>724936154033605</t>
+          <t>1412353528623168</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>1374769798168339</t>
+          <t>28796808946621878</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Upload your resume</t>
+          <t>FPA AI | Enterprise Technology &amp; AI Advisory | Join US! | In Digital Transformation | Of Our Offerings | Scan QR</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr"/>
       <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="7" t="n">
-        <v>46277.85913194445</v>
+        <v>46292.20268518518</v>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>General IT job seekers</t>
+          <t>Consulting / architecture talent (closest match to Zarthi)</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Direct response (CV upload)</t>
+          <t>Employer brand + offerings</t>
         </is>
       </c>
       <c r="M10" s="8" t="inlineStr">
@@ -984,38 +984,38 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Technopark, Trivandrum</t>
+          <t>Exano Technologies</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>140899789320354</t>
+          <t>724936154033605</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>2217098326355842</t>
+          <t>1374769798168339</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>(no headline returned)</t>
+          <t>Upload your resume</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr"/>
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="7" t="n">
-        <v>46284.49287037037</v>
+        <v>46277.85913194445</v>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Trivandrum tech workforce (one of Zarthi's 3 locations)</t>
+          <t>General IT job seekers</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Tech-park community</t>
+          <t>Direct response (CV upload)</t>
         </is>
       </c>
       <c r="M11" s="8" t="inlineStr">
@@ -1035,43 +1035,43 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>B · Same audience</t>
+          <t>A · Hiring ad</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>EdYoda</t>
+          <t>Technopark, Trivandrum</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>813649275509075</t>
+          <t>140899789320354</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>1443197407729118</t>
+          <t>2217098326355842</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Become a CERTIFIED MULTICLOUD ARCHITECT</t>
+          <t>(no headline returned)</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr"/>
       <c r="H12" s="6" t="inlineStr"/>
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="7" t="n">
-        <v>46293.65880787037</v>
+        <v>46284.49287037037</v>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>Engineers wanting multi-cloud architect roles</t>
+          <t>Trivandrum tech workforce (one of Zarthi's 3 locations)</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Certification / upskilling</t>
+          <t>Tech-park community</t>
         </is>
       </c>
       <c r="M12" s="8" t="inlineStr">
@@ -1096,38 +1096,38 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>R9ST IT Academy</t>
+          <t>EdYoda</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>484287398101280</t>
+          <t>813649275509075</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>2769022723493673</t>
+          <t>1443197407729118</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Live AWS Solutions Architect Training</t>
+          <t>Become a CERTIFIED MULTICLOUD ARCHITECT</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr"/>
       <c r="H13" s="6" t="inlineStr"/>
       <c r="I13" s="6" t="inlineStr"/>
       <c r="J13" s="7" t="n">
-        <v>46293.65517361111</v>
+        <v>46293.65880787037</v>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>AWS engineers moving into architecture</t>
+          <t>Engineers wanting multi-cloud architect roles</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Certification / upskilling</t>
         </is>
       </c>
       <c r="M13" s="8" t="inlineStr">
@@ -1152,38 +1152,38 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Software System Design / Architecture Interview</t>
+          <t>R9ST IT Academy</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>166719546523044</t>
+          <t>484287398101280</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>1644512954128194</t>
+          <t>2769022723493673</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Become a Strong Software Architect</t>
+          <t>Live AWS Solutions Architect Training</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr"/>
       <c r="H14" s="6" t="inlineStr"/>
       <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="7" t="n">
-        <v>46293.56111111111</v>
+        <v>46293.65517361111</v>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>Engineers preparing for architect interviews</t>
+          <t>AWS engineers moving into architecture</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Interview prep</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="M14" s="8" t="inlineStr">
@@ -1208,38 +1208,38 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Console Flare</t>
+          <t>Software System Design / Architecture Interview</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>331465344179561</t>
+          <t>166719546523044</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>1584154803195990</t>
+          <t>1644512954128194</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>For Working Professionals Only</t>
+          <t>Become a Strong Software Architect</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr"/>
       <c r="H15" s="6" t="inlineStr"/>
       <c r="I15" s="6" t="inlineStr"/>
       <c r="J15" s="7" t="n">
-        <v>46293.60974537037</v>
+        <v>46293.56111111111</v>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Experienced working professionals</t>
+          <t>Engineers preparing for architect interviews</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Exclusivity call-out</t>
+          <t>Interview prep</t>
         </is>
       </c>
       <c r="M15" s="8" t="inlineStr">
@@ -1264,29 +1264,29 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>GUVI</t>
+          <t>Console Flare</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>386984684662653</t>
+          <t>331465344179561</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>1059681169841736</t>
+          <t>1584154803195990</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Only For Working Professionals</t>
+          <t>For Working Professionals Only</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr"/>
       <c r="I16" s="6" t="inlineStr"/>
       <c r="J16" s="7" t="n">
-        <v>46239.39222222222</v>
+        <v>46293.60974537037</v>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
@@ -1320,38 +1320,38 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Sprinted - Software Services</t>
+          <t>GUVI</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>1276977545488723</t>
+          <t>386984684662653</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>1857077995471994</t>
+          <t>1059681169841736</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Become an AI-First Data Engineer | Switch to Product-Based Companies</t>
+          <t>Only For Working Professionals</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr"/>
       <c r="H17" s="6" t="inlineStr"/>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="7" t="n">
-        <v>46289.75611111111</v>
+        <v>46239.39222222222</v>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>IT services staff wanting to move to product companies</t>
+          <t>Experienced working professionals</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Career-switch motive</t>
+          <t>Exclusivity call-out</t>
         </is>
       </c>
       <c r="M17" s="8" t="inlineStr">
@@ -1376,38 +1376,38 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Nexverse Learning</t>
+          <t>Sprinted - Software Services</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>591969314010473</t>
+          <t>1276977545488723</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>1493454822791932</t>
+          <t>1857077995471994</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Don't Just Learn DevOps. Become Production-Ready.</t>
+          <t>Become an AI-First Data Engineer | Switch to Product-Based Companies</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr"/>
       <c r="H18" s="6" t="inlineStr"/>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="7" t="n">
-        <v>46292.09815972222</v>
+        <v>46289.75611111111</v>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>DevOps engineers</t>
+          <t>IT services staff wanting to move to product companies</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Contrast hook</t>
+          <t>Career-switch motive</t>
         </is>
       </c>
       <c r="M18" s="8" t="inlineStr">
@@ -1432,93 +1432,149 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Open Source India</t>
+          <t>Nexverse Learning</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>296874510990</t>
+          <t>591969314010473</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>1758578985420711</t>
+          <t>1493454822791932</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Built to Scale | DuckDB engine for MariaDB | Data Architecture for Agentic AI Systems</t>
+          <t>Don't Just Learn DevOps. Become Production-Ready.</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr"/>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="7" t="n">
+        <v>46292.09815972222</v>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>DevOps engineers</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Contrast hook</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>Open ad</t>
+        </is>
+      </c>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>INR</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>B · Same audience</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Open Source India</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>296874510990</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>1758578985420711</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Built to Scale | DuckDB engine for MariaDB | Data Architecture for Agentic AI Systems</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="7" t="n">
         <v>46293.60177083333</v>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Architects and senior engineers (tech conference)</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Event / thought leadership</t>
         </is>
       </c>
-      <c r="M19" s="8" t="inlineStr">
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>Open ad</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="N20" s="4" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Hiring ads</t>
-        </is>
-      </c>
-      <c r="C22" s="10">
-        <f>COUNTIF(B5:B19,"A*")</f>
-        <v/>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>Same-audience ads</t>
+          <t>Hiring ads</t>
         </is>
       </c>
       <c r="C23" s="10">
-        <f>COUNTIF(B5:B19,"B*")</f>
+        <f>COUNTIF(B5:B20,"A*")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="10" t="inlineStr">
         <is>
+          <t>Same-audience ads</t>
+        </is>
+      </c>
+      <c r="C24" s="10">
+        <f>COUNTIF(B5:B20,"B*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="10" t="inlineStr">
+        <is>
           <t>Captions filled in</t>
         </is>
       </c>
-      <c r="C24" s="10">
-        <f>COUNTA(G5:G19)&amp;" of "&amp;COUNTA(E5:E19)</f>
+      <c r="C25" s="10">
+        <f>COUNTA(G5:G20)&amp;" of "&amp;COUNTA(E5:E20)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N19"/>
+  <autoFilter ref="A4:N20"/>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
   </mergeCells>
@@ -1538,6 +1594,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Add caption, CTA and format for Software System Design ad from Ad Library
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDCiezjHZtSKU1uv8fZ38q
</commit_message>
<xml_diff>
--- a/deliverables/Zarthi_Competitor_Meta_Ads_India.xlsx
+++ b/deliverables/Zarthi_Competitor_Meta_Ads_India.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Takeaways for Zarthi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Competitor Ads'!$A$4:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Competitor Ads'!$A$4:$O$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -541,7 +541,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -549,6 +549,7 @@
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,7 +562,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Pulled 28 Sep 2026 from Meta Ad Library, filtered to ads delivered in India, active, paid in INR. Caption, Description and CTA (yellow) are not returned by Meta's Ad Library tool, and facebook.com is blocked from this environment. Open the link in each row to view them.</t>
+          <t>Pulled 28 Sep 2026 from Meta Ad Library, filtered to ads delivered in India, active, paid in INR. Caption, Description and CTA (yellow) are not returned by Meta's Ad Library tool, and facebook.com is blocked from this environment. Filled rows were copied from the Ad Library page (screenshot supplied by Zarthi team); yellow cells are still to fill.</t>
         </is>
       </c>
     </row>
@@ -634,6 +635,11 @@
       <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Currency</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Format / on-image text</t>
         </is>
       </c>
     </row>
@@ -692,6 +698,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -748,6 +755,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -804,6 +812,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -860,6 +869,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -916,6 +926,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -972,6 +983,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -1028,6 +1040,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -1084,6 +1097,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1140,6 +1154,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -1196,6 +1211,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1226,9 +1242,21 @@
           <t>Become a Strong Software Architect</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr"/>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Software Architects don't just earn more they think differently. Don't Code throughout the year and call yourself an Architect, you're a Senior Software Engineer not an Architect. Become a Real Software Architect with this course. / “This Training is Only for 10+ Years Software Engineers | Limited Batch | Serious Learners Only”. Training has AI and cloud also as one package and cloud and ai is also present and optional. All classes are live and recorded also. … (truncated in Ad Library)</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>None shown (card headline: 'Become an Strong Software Architect', link fb.me)</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Apply Now</t>
+        </is>
+      </c>
       <c r="J15" s="7" t="n">
         <v>46293.56111111111</v>
       </c>
@@ -1250,6 +1278,11 @@
       <c r="N15" s="4" t="inlineStr">
         <is>
           <t>INR</t>
+        </is>
+      </c>
+      <c r="O15" s="4" t="inlineStr">
+        <is>
+          <t>Carousel (3+ cards) · link: fb.me. Card 1 image: 'Software Architects Don't Just Earn More - They Think Differently. Learn How?!' Card 2 image: 'Dont Be a Coder or Designer - Be a Software Architect with AI Knowledge · Join Software Architect, System Design and AI Training (ALL in Great packages)' (Flying stocks technologies). Card 3: 'Code… Architect… Think… Software Architect… REGISTER'</t>
         </is>
       </c>
     </row>
@@ -1308,6 +1341,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -1364,6 +1398,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -1420,6 +1455,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -1476,6 +1512,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -1532,6 +1569,7 @@
           <t>INR</t>
         </is>
       </c>
+      <c r="O20" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -1574,9 +1612,9 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N20"/>
+  <autoFilter ref="A4:O20"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A2:O2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId1"/>
@@ -1653,7 +1691,7 @@
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>Hiring ads that do run put years in the headline (7+, 6–8, 6+).</t>
+          <t>Hiring ads that do run put years in the headline (7+, 6–8, 6+). Even the architect course ad says ‘Only for 10+ Years Software Engineers’.</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">

</xml_diff>